<commit_message>
replacing vapply(MSEAres$leadingEdge, length) with vapply(MSEAres$leadingEdge, length, integer(1))
</commit_message>
<xml_diff>
--- a/vignettes/gsea_results.xlsx
+++ b/vignettes/gsea_results.xlsx
@@ -41,18 +41,18 @@
     <t xml:space="preserve">input_count</t>
   </si>
   <si>
+    <t xml:space="preserve">Biosynthesis_of_amino_acids</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C00074, C00079, C00065, C00123, C00148, C00026, C00082, C00263, C00022, C00152, C00041</t>
+  </si>
+  <si>
     <t xml:space="preserve">Central_carbon_metabolism_in_cancer</t>
   </si>
   <si>
     <t xml:space="preserve">C00074, C00079, C00065, C00123, C00148, C00026, C00082, C00022, C00152, C00041</t>
   </si>
   <si>
-    <t xml:space="preserve">Biosynthesis_of_amino_acids</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C00074, C00079, C00065, C00123, C00148, C00026, C00082, C00263, C00022, C00152, C00041</t>
-  </si>
-  <si>
     <t xml:space="preserve">Metabolic_pathways</t>
   </si>
   <si>
@@ -65,15 +65,15 @@
     <t xml:space="preserve">C00074, C00065, C00295, C01909, C06423, C00105, C00026, C00082, C00051, C00022, C00127, C00015, C00153, C00328, C00314, C00049</t>
   </si>
   <si>
+    <t xml:space="preserve">Aminoacyl-tRNA_biosynthesis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C00079, C00065, C00123, C00148, C00082, C00152, C00041</t>
+  </si>
+  <si>
     <t xml:space="preserve">Protein_digestion_and_absorption</t>
   </si>
   <si>
-    <t xml:space="preserve">C00079, C00065, C00123, C00148, C00082, C00152, C00041</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aminoacyl-tRNA_biosynthesis</t>
-  </si>
-  <si>
     <t xml:space="preserve">D-Amino_acid_metabolism</t>
   </si>
   <si>
@@ -128,16 +128,16 @@
     <t xml:space="preserve">C00074, C00065, C00026, C00022, C00041, C00049, C00048, C01005</t>
   </si>
   <si>
+    <t xml:space="preserve">Glyoxylate_and_dicarboxylate_metabolism</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C00065, C00026, C00022</t>
+  </si>
+  <si>
     <t xml:space="preserve">Purine_metabolism</t>
   </si>
   <si>
     <t xml:space="preserve">C00242, C00366, C00385, C00144, C00035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glyoxylate_and_dicarboxylate_metabolism</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C00065, C00026, C00022</t>
   </si>
   <si>
     <t xml:space="preserve">beta-Alanine_metabolism</t>
@@ -518,28 +518,28 @@
         <v>9</v>
       </c>
       <c r="B2" t="n">
-        <v>0.00213852073225541</v>
+        <v>0.00165578714870562</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0339862481681217</v>
+        <v>0.0228687735252716</v>
       </c>
       <c r="D2" t="n">
-        <v>0.431707695803346</v>
+        <v>0.45505986738723</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.659381219971923</v>
+        <v>-0.587907678501511</v>
       </c>
       <c r="F2" t="n">
-        <v>-1.81009923433636</v>
+        <v>-1.83725681215786</v>
       </c>
       <c r="G2" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H2" t="s">
         <v>10</v>
       </c>
       <c r="I2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -547,28 +547,28 @@
         <v>11</v>
       </c>
       <c r="B3" t="n">
-        <v>0.00339862481681218</v>
+        <v>0.00228687735252716</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0339862481681217</v>
+        <v>0.0228687735252716</v>
       </c>
       <c r="D3" t="n">
         <v>0.431707695803346</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.587907678501511</v>
+        <v>-0.659381219971923</v>
       </c>
       <c r="F3" t="n">
-        <v>-1.80324944160328</v>
+        <v>-1.84281532636888</v>
       </c>
       <c r="G3" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="H3" t="s">
         <v>12</v>
       </c>
       <c r="I3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -576,10 +576,10 @@
         <v>13</v>
       </c>
       <c r="B4" t="n">
-        <v>0.00931935923904676</v>
+        <v>0.00970646999465802</v>
       </c>
       <c r="C4" t="n">
-        <v>0.062129061593645</v>
+        <v>0.0526860830838493</v>
       </c>
       <c r="D4" t="n">
         <v>0.380730400722792</v>
@@ -588,7 +588,7 @@
         <v>-0.347062010834737</v>
       </c>
       <c r="F4" t="n">
-        <v>-1.45505795843938</v>
+        <v>-1.44556264115556</v>
       </c>
       <c r="G4" t="n">
         <v>148</v>
@@ -605,19 +605,19 @@
         <v>15</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0246813757895584</v>
+        <v>0.0116749754531019</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0830689215728985</v>
+        <v>0.0526860830838493</v>
       </c>
       <c r="D5" t="n">
-        <v>0.352487857583619</v>
+        <v>0.380730400722792</v>
       </c>
       <c r="E5" t="n">
         <v>-0.477675319380464</v>
       </c>
       <c r="F5" t="n">
-        <v>-1.61413017033871</v>
+        <v>-1.61574308775682</v>
       </c>
       <c r="G5" t="n">
         <v>33</v>
@@ -634,22 +634,22 @@
         <v>17</v>
       </c>
       <c r="B6" t="n">
-        <v>0.0269787491790036</v>
+        <v>0.0131715207709623</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0830689215728985</v>
+        <v>0.0526860830838493</v>
       </c>
       <c r="D6" t="n">
-        <v>0.352487857583619</v>
+        <v>0.380730400722792</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.595792599572215</v>
+        <v>-0.646558608064039</v>
       </c>
       <c r="F6" t="n">
-        <v>-1.55630884410164</v>
+        <v>-1.66636016576768</v>
       </c>
       <c r="G6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H6" t="s">
         <v>18</v>
@@ -663,22 +663,22 @@
         <v>19</v>
       </c>
       <c r="B7" t="n">
-        <v>0.0284225686550338</v>
+        <v>0.0260597243704394</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0830689215728985</v>
+        <v>0.0783141639184488</v>
       </c>
       <c r="D7" t="n">
         <v>0.352487857583619</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.646558608064039</v>
+        <v>-0.595792599572215</v>
       </c>
       <c r="F7" t="n">
-        <v>-1.60376383443085</v>
+        <v>-1.60022173382044</v>
       </c>
       <c r="G7" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H7" t="s">
         <v>18</v>
@@ -692,10 +692,10 @@
         <v>20</v>
       </c>
       <c r="B8" t="n">
-        <v>0.0290741225505145</v>
+        <v>0.0274099573714571</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0830689215728985</v>
+        <v>0.0783141639184488</v>
       </c>
       <c r="D8" t="n">
         <v>0.352487857583619</v>
@@ -704,7 +704,7 @@
         <v>-0.592515268437193</v>
       </c>
       <c r="F8" t="n">
-        <v>-1.5477479129418</v>
+        <v>-1.59141924699037</v>
       </c>
       <c r="G8" t="n">
         <v>13</v>
@@ -721,19 +721,19 @@
         <v>22</v>
       </c>
       <c r="B9" t="n">
-        <v>0.068904593639576</v>
+        <v>0.0598911070780399</v>
       </c>
       <c r="C9" t="n">
-        <v>0.17226148409894</v>
+        <v>0.1497277676951</v>
       </c>
       <c r="D9" t="n">
-        <v>0.227987202850442</v>
+        <v>0.248911114434702</v>
       </c>
       <c r="E9" t="n">
         <v>-0.580512907394844</v>
       </c>
       <c r="F9" t="n">
-        <v>-1.43994000650277</v>
+        <v>-1.49614214787616</v>
       </c>
       <c r="G9" t="n">
         <v>11</v>
@@ -750,19 +750,19 @@
         <v>24</v>
       </c>
       <c r="B10" t="n">
-        <v>0.139616055846422</v>
+        <v>0.117857142857143</v>
       </c>
       <c r="C10" t="n">
-        <v>0.272938443670151</v>
+        <v>0.225631768953069</v>
       </c>
       <c r="D10" t="n">
-        <v>0.155241966228839</v>
+        <v>0.172324344900946</v>
       </c>
       <c r="E10" t="n">
         <v>-0.4947670412642</v>
       </c>
       <c r="F10" t="n">
-        <v>-1.35820890168108</v>
+        <v>-1.38275743834905</v>
       </c>
       <c r="G10" t="n">
         <v>15</v>
@@ -779,19 +779,19 @@
         <v>26</v>
       </c>
       <c r="B11" t="n">
-        <v>0.144876325088339</v>
+        <v>0.121597096188748</v>
       </c>
       <c r="C11" t="n">
-        <v>0.272938443670151</v>
+        <v>0.225631768953069</v>
       </c>
       <c r="D11" t="n">
-        <v>0.153158808683073</v>
+        <v>0.170932335370056</v>
       </c>
       <c r="E11" t="n">
         <v>-0.532292492269077</v>
       </c>
       <c r="F11" t="n">
-        <v>-1.32033111583854</v>
+        <v>-1.37186481564335</v>
       </c>
       <c r="G11" t="n">
         <v>11</v>
@@ -808,19 +808,19 @@
         <v>28</v>
       </c>
       <c r="B12" t="n">
-        <v>0.15979381443299</v>
+        <v>0.132978723404255</v>
       </c>
       <c r="C12" t="n">
-        <v>0.272938443670151</v>
+        <v>0.225631768953069</v>
       </c>
       <c r="D12" t="n">
-        <v>0.142901149386948</v>
+        <v>0.160801401070022</v>
       </c>
       <c r="E12" t="n">
         <v>-0.414742469888983</v>
       </c>
       <c r="F12" t="n">
-        <v>-1.28440570918313</v>
+        <v>-1.30522269154083</v>
       </c>
       <c r="G12" t="n">
         <v>24</v>
@@ -837,19 +837,19 @@
         <v>30</v>
       </c>
       <c r="B13" t="n">
-        <v>0.163763066202091</v>
+        <v>0.135379061371841</v>
       </c>
       <c r="C13" t="n">
-        <v>0.272938443670151</v>
+        <v>0.225631768953069</v>
       </c>
       <c r="D13" t="n">
-        <v>0.142056643575821</v>
+        <v>0.160801401070022</v>
       </c>
       <c r="E13" t="n">
         <v>-0.502026269104197</v>
       </c>
       <c r="F13" t="n">
-        <v>-1.31137567525881</v>
+        <v>-1.34837751819365</v>
       </c>
       <c r="G13" t="n">
         <v>13</v>
@@ -866,19 +866,19 @@
         <v>32</v>
       </c>
       <c r="B14" t="n">
-        <v>0.181818181818182</v>
+        <v>0.154804270462633</v>
       </c>
       <c r="C14" t="n">
-        <v>0.27972027972028</v>
+        <v>0.238160416096359</v>
       </c>
       <c r="D14" t="n">
-        <v>0.132846300606183</v>
+        <v>0.148261500475107</v>
       </c>
       <c r="E14" t="n">
         <v>-0.406841097924122</v>
       </c>
       <c r="F14" t="n">
-        <v>-1.24787617083497</v>
+        <v>-1.27140979095913</v>
       </c>
       <c r="G14" t="n">
         <v>23</v>
@@ -895,19 +895,19 @@
         <v>34</v>
       </c>
       <c r="B15" t="n">
-        <v>0.250871080139373</v>
+        <v>0.194945848375451</v>
       </c>
       <c r="C15" t="n">
-        <v>0.356643356643357</v>
+        <v>0.278494069107788</v>
       </c>
       <c r="D15" t="n">
-        <v>0.11146266692298</v>
+        <v>0.131457611642763</v>
       </c>
       <c r="E15" t="n">
         <v>-0.463564343022208</v>
       </c>
       <c r="F15" t="n">
-        <v>-1.21090676079837</v>
+        <v>-1.24507376771876</v>
       </c>
       <c r="G15" t="n">
         <v>13</v>
@@ -924,19 +924,19 @@
         <v>36</v>
       </c>
       <c r="B16" t="n">
-        <v>0.267482517482518</v>
+        <v>0.25</v>
       </c>
       <c r="C16" t="n">
-        <v>0.356643356643357</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="D16" t="n">
-        <v>0.107554375265169</v>
+        <v>0.112843355675562</v>
       </c>
       <c r="E16" t="n">
         <v>-0.410921588850623</v>
       </c>
       <c r="F16" t="n">
-        <v>-1.15735320979748</v>
+        <v>-1.16063362033024</v>
       </c>
       <c r="G16" t="n">
         <v>16</v>
@@ -953,28 +953,28 @@
         <v>38</v>
       </c>
       <c r="B17" t="n">
-        <v>0.316254416961131</v>
+        <v>0.291208791208791</v>
       </c>
       <c r="C17" t="n">
-        <v>0.379901960784314</v>
+        <v>0.345154161843628</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0978773277424561</v>
+        <v>0.105125131597001</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.372136175420514</v>
+        <v>-0.461753679537052</v>
       </c>
       <c r="F17" t="n">
-        <v>-1.10574177108158</v>
+        <v>-1.15550149364592</v>
       </c>
       <c r="G17" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H17" t="s">
         <v>39</v>
       </c>
       <c r="I17" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -982,28 +982,28 @@
         <v>40</v>
       </c>
       <c r="B18" t="n">
-        <v>0.322916666666667</v>
+        <v>0.293381037567084</v>
       </c>
       <c r="C18" t="n">
-        <v>0.379901960784314</v>
+        <v>0.345154161843628</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0956031492204301</v>
+        <v>0.103197466945307</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.461753679537052</v>
+        <v>-0.372136175420514</v>
       </c>
       <c r="F18" t="n">
-        <v>-1.12092868434192</v>
+        <v>-1.11914327135785</v>
       </c>
       <c r="G18" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H18" t="s">
         <v>41</v>
       </c>
       <c r="I18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
@@ -1011,19 +1011,19 @@
         <v>42</v>
       </c>
       <c r="B19" t="n">
-        <v>0.511737089201878</v>
+        <v>0.474835886214442</v>
       </c>
       <c r="C19" t="n">
-        <v>0.568596765779864</v>
+        <v>0.527595429127158</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0865399737444125</v>
+        <v>0.086794975677172</v>
       </c>
       <c r="E19" t="n">
         <v>0.376554907494225</v>
       </c>
       <c r="F19" t="n">
-        <v>0.959723808419876</v>
+        <v>0.98342227166151</v>
       </c>
       <c r="G19" t="n">
         <v>10</v>
@@ -1040,19 +1040,19 @@
         <v>44</v>
       </c>
       <c r="B20" t="n">
-        <v>0.933682373472949</v>
+        <v>0.921428571428571</v>
       </c>
       <c r="C20" t="n">
-        <v>0.980902777777778</v>
+        <v>0.969924812030075</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0425877779273254</v>
+        <v>0.0442407423477375</v>
       </c>
       <c r="E20" t="n">
         <v>-0.218104455582059</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.598729075224866</v>
+        <v>-0.609550623102479</v>
       </c>
       <c r="G20" t="n">
         <v>15</v>
@@ -1069,19 +1069,19 @@
         <v>46</v>
       </c>
       <c r="B21" t="n">
-        <v>0.980902777777778</v>
+        <v>0.987179487179487</v>
       </c>
       <c r="C21" t="n">
-        <v>0.980902777777778</v>
+        <v>0.987179487179487</v>
       </c>
       <c r="D21" t="n">
-        <v>0.0400845633477088</v>
+        <v>0.0422468188360053</v>
       </c>
       <c r="E21" t="n">
         <v>-0.201096271807338</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.488170618605708</v>
+        <v>-0.503227267561731</v>
       </c>
       <c r="G21" t="n">
         <v>10</v>

</xml_diff>